<commit_message>
initial Add testwp functions
</commit_message>
<xml_diff>
--- a/inst/extdata/example_test_wp.xlsx
+++ b/inst/extdata/example_test_wp.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="36">
   <si>
     <t>VISIT</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -116,10 +116,6 @@
     <t>生命体征</t>
   </si>
   <si>
-    <t>RD(-7d)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>EX(≤24h)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -131,10 +127,6 @@
     <t>血常规</t>
   </si>
   <si>
-    <t>RD(0)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>血生化</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -151,6 +143,22 @@
   </si>
   <si>
     <t>EX(0)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FD(0)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FD(-7d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>FD(-7d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EX(≤1d)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -531,16 +539,16 @@
         <v>23</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E1" t="s">
         <v>27</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -559,19 +567,19 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="G3" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -582,10 +590,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -596,10 +604,10 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -610,10 +618,10 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -624,19 +632,19 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -647,10 +655,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -661,10 +669,10 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -675,10 +683,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -689,19 +697,19 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -712,10 +720,10 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -726,10 +734,10 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -740,19 +748,19 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -763,19 +771,19 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D15" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -786,10 +794,10 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -800,10 +808,10 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D17" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -814,19 +822,19 @@
         <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D18" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E18" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -837,10 +845,10 @@
         <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -851,10 +859,10 @@
         <v>19</v>
       </c>
       <c r="C20" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="D20" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -865,19 +873,19 @@
         <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G21" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -888,20 +896,21 @@
         <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F22" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add window type: prev-h/prev-d
</commit_message>
<xml_diff>
--- a/inst/extdata/example_test_wp.xlsx
+++ b/inst/extdata/example_test_wp.xlsx
@@ -4,11 +4,15 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="QL0911-302" sheetId="1" r:id="rId1"/>
+    <sheet name="QLS31905-301" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'QLS31905-301'!$A$1:$F$99</definedName>
+  </definedNames>
   <calcPr calcId="162913" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -19,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="244">
   <si>
     <t>VISIT</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -116,6 +120,10 @@
     <t>生命体征</t>
   </si>
   <si>
+    <t>RD(-7d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>EX(≤24h)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -127,6 +135,10 @@
     <t>血常规</t>
   </si>
   <si>
+    <t>RD(0)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>血生化</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -146,19 +158,643 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>FD(0)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>FD(-7d)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>FD(-7d)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
+    <t>筛选期</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>预激访视</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>C1D1</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>C1D8</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>C2D1</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>C2D8</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>C3D1</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>C3D8</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>C4D1</t>
+  </si>
+  <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t>C4D8</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>C5D1</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>C5D8</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>C6D1</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>C6D8</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>C7D1</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>C7D8</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>C8D1</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>C8D8</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>C9D1</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>C9D8</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>C10D1</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>C10D8</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>C11D1</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>C11D8</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>C12D1</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>C12D8</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>C13D1</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>C13D8</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>C14D1</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>C14D8</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>C15D1</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>C15D8</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>C16D1</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>C16D8</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>C17D1</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>C17D8</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>C18D1</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>C18D8</t>
+  </si>
+  <si>
+    <t>39</t>
+  </si>
+  <si>
+    <t>C19D1</t>
+  </si>
+  <si>
+    <t>40</t>
+  </si>
+  <si>
+    <t>C19D8</t>
+  </si>
+  <si>
+    <t>41</t>
+  </si>
+  <si>
+    <t>C20D1</t>
+  </si>
+  <si>
+    <t>42</t>
+  </si>
+  <si>
+    <t>C20D8</t>
+  </si>
+  <si>
+    <t>43</t>
+  </si>
+  <si>
+    <t>C21D1</t>
+  </si>
+  <si>
+    <t>44</t>
+  </si>
+  <si>
+    <t>C21D8</t>
+  </si>
+  <si>
+    <t>45</t>
+  </si>
+  <si>
+    <t>C22D1</t>
+  </si>
+  <si>
+    <t>46</t>
+  </si>
+  <si>
+    <t>C22D8</t>
+  </si>
+  <si>
+    <t>47</t>
+  </si>
+  <si>
+    <t>C23D1</t>
+  </si>
+  <si>
+    <t>48</t>
+  </si>
+  <si>
+    <t>C23D8</t>
+  </si>
+  <si>
+    <t>49</t>
+  </si>
+  <si>
+    <t>C24D1</t>
+  </si>
+  <si>
+    <t>50</t>
+  </si>
+  <si>
+    <t>C24D8</t>
+  </si>
+  <si>
+    <t>51</t>
+  </si>
+  <si>
+    <t>C25D1</t>
+  </si>
+  <si>
+    <t>52</t>
+  </si>
+  <si>
+    <t>C25D8</t>
+  </si>
+  <si>
+    <t>53</t>
+  </si>
+  <si>
+    <t>C26D1</t>
+  </si>
+  <si>
+    <t>54</t>
+  </si>
+  <si>
+    <t>C26D8</t>
+  </si>
+  <si>
+    <t>55</t>
+  </si>
+  <si>
+    <t>C27D1</t>
+  </si>
+  <si>
+    <t>56</t>
+  </si>
+  <si>
+    <t>C27D8</t>
+  </si>
+  <si>
+    <t>57</t>
+  </si>
+  <si>
+    <t>C28D1</t>
+  </si>
+  <si>
+    <t>58</t>
+  </si>
+  <si>
+    <t>C28D8</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>C29D1</t>
+  </si>
+  <si>
+    <t>60</t>
+  </si>
+  <si>
+    <t>C29D8</t>
+  </si>
+  <si>
+    <t>61</t>
+  </si>
+  <si>
+    <t>C30D1</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>C30D8</t>
+  </si>
+  <si>
+    <t>63</t>
+  </si>
+  <si>
+    <t>C31D1</t>
+  </si>
+  <si>
+    <t>64</t>
+  </si>
+  <si>
+    <t>C31D8</t>
+  </si>
+  <si>
+    <t>65</t>
+  </si>
+  <si>
+    <t>C32D1</t>
+  </si>
+  <si>
+    <t>66</t>
+  </si>
+  <si>
+    <t>C32D8</t>
+  </si>
+  <si>
+    <t>67</t>
+  </si>
+  <si>
+    <t>C33D1</t>
+  </si>
+  <si>
+    <t>68</t>
+  </si>
+  <si>
+    <t>C33D8</t>
+  </si>
+  <si>
+    <t>69</t>
+  </si>
+  <si>
+    <t>C34D1</t>
+  </si>
+  <si>
+    <t>70</t>
+  </si>
+  <si>
+    <t>C34D8</t>
+  </si>
+  <si>
+    <t>71</t>
+  </si>
+  <si>
+    <t>C35D1</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>C35D8</t>
+  </si>
+  <si>
+    <t>73</t>
+  </si>
+  <si>
+    <t>C36D1</t>
+  </si>
+  <si>
+    <t>74</t>
+  </si>
+  <si>
+    <t>C36D8</t>
+  </si>
+  <si>
+    <t>75</t>
+  </si>
+  <si>
+    <t>C37D1</t>
+  </si>
+  <si>
+    <t>76</t>
+  </si>
+  <si>
+    <t>C37D8</t>
+  </si>
+  <si>
+    <t>77</t>
+  </si>
+  <si>
+    <t>C38D1</t>
+  </si>
+  <si>
+    <t>78</t>
+  </si>
+  <si>
+    <t>C38D8</t>
+  </si>
+  <si>
+    <t>79</t>
+  </si>
+  <si>
+    <t>C39D1</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>C39D8</t>
+  </si>
+  <si>
+    <t>81</t>
+  </si>
+  <si>
+    <t>C40D1</t>
+  </si>
+  <si>
+    <t>82</t>
+  </si>
+  <si>
+    <t>C40D8</t>
+  </si>
+  <si>
+    <t>83</t>
+  </si>
+  <si>
+    <t>C41D1</t>
+  </si>
+  <si>
+    <t>84</t>
+  </si>
+  <si>
+    <t>C41D8</t>
+  </si>
+  <si>
+    <t>85</t>
+  </si>
+  <si>
+    <t>C42D1</t>
+  </si>
+  <si>
+    <t>86</t>
+  </si>
+  <si>
+    <t>C42D8</t>
+  </si>
+  <si>
+    <t>87</t>
+  </si>
+  <si>
+    <t>C43D1</t>
+  </si>
+  <si>
+    <t>88</t>
+  </si>
+  <si>
+    <t>C43D8</t>
+  </si>
+  <si>
+    <t>89</t>
+  </si>
+  <si>
+    <t>C44D1</t>
+  </si>
+  <si>
+    <t>90</t>
+  </si>
+  <si>
+    <t>C44D8</t>
+  </si>
+  <si>
+    <t>91</t>
+  </si>
+  <si>
+    <t>C45D1</t>
+  </si>
+  <si>
+    <t>92</t>
+  </si>
+  <si>
+    <t>C45D8</t>
+  </si>
+  <si>
+    <t>93</t>
+  </si>
+  <si>
+    <t>治疗结束/提前退出</t>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>安全性随访-末次用药30天</t>
+  </si>
+  <si>
+    <t>142</t>
+  </si>
+  <si>
+    <t>安全性随访-末次用药60天</t>
+  </si>
+  <si>
+    <t>143</t>
+  </si>
+  <si>
+    <t>安全性随访-末次用药90天</t>
+  </si>
+  <si>
+    <t>144</t>
+  </si>
+  <si>
+    <t>生存随访</t>
+  </si>
+  <si>
+    <t>146</t>
+  </si>
+  <si>
+    <t>研究结束</t>
+  </si>
+  <si>
+    <t>147</t>
+  </si>
+  <si>
+    <t>生命体征/血氧饱和度</t>
+  </si>
+  <si>
+    <t>SV(±1d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>体重</t>
   </si>
   <si>
     <t>EX(≤1d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EX(≤3d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EX(≤2d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>血常规</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>尿常规</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>12-导联心电图</t>
+  </si>
+  <si>
+    <t>12-导联心电图（筛选期）</t>
+  </si>
+  <si>
+    <t>EX(prev-h)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EX(PREV-h)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EX(PREV-d)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>EX(prev-H)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -227,7 +863,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -238,6 +874,9 @@
     </xf>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -539,16 +1178,16 @@
         <v>23</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -567,19 +1206,19 @@
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="G3" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -590,10 +1229,10 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -604,10 +1243,10 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -618,10 +1257,10 @@
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -632,19 +1271,19 @@
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -655,10 +1294,10 @@
         <v>7</v>
       </c>
       <c r="C8" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -669,10 +1308,10 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -683,10 +1322,10 @@
         <v>9</v>
       </c>
       <c r="C10" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -697,19 +1336,19 @@
         <v>10</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D11" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
@@ -720,10 +1359,10 @@
         <v>11</v>
       </c>
       <c r="C12" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
@@ -734,10 +1373,10 @@
         <v>12</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D13" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
@@ -748,19 +1387,19 @@
         <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
@@ -771,19 +1410,19 @@
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
@@ -794,10 +1433,10 @@
         <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
@@ -808,10 +1447,10 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
@@ -822,19 +1461,19 @@
         <v>17</v>
       </c>
       <c r="C18" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E18" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
@@ -845,10 +1484,10 @@
         <v>18</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
@@ -859,10 +1498,10 @@
         <v>19</v>
       </c>
       <c r="C20" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
@@ -873,19 +1512,19 @@
         <v>20</v>
       </c>
       <c r="C21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G21" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
@@ -896,19 +1535,2009 @@
         <v>21</v>
       </c>
       <c r="C22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H99"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="24.77734375" customWidth="1"/>
+    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+    <col min="3" max="3" width="23.88671875" customWidth="1"/>
+    <col min="7" max="7" width="20.5546875" customWidth="1"/>
+    <col min="8" max="8" width="14.88671875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="E1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F1" t="s">
+        <v>237</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>240</v>
+      </c>
+      <c r="D3" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" t="s">
+        <v>241</v>
+      </c>
+      <c r="D4" t="s">
+        <v>234</v>
+      </c>
+      <c r="E4" t="s">
+        <v>234</v>
+      </c>
+      <c r="F4" t="s">
+        <v>234</v>
+      </c>
+      <c r="H4" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
+        <v>242</v>
+      </c>
+      <c r="D5" t="s">
+        <v>235</v>
+      </c>
+      <c r="E5" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" t="s">
+        <v>243</v>
+      </c>
+      <c r="D6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E6" t="s">
+        <v>234</v>
+      </c>
+      <c r="F6" t="s">
+        <v>234</v>
+      </c>
+      <c r="H6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D7" t="s">
+        <v>235</v>
+      </c>
+      <c r="E7" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C8" t="s">
+        <v>240</v>
+      </c>
+      <c r="D8" t="s">
+        <v>234</v>
+      </c>
+      <c r="E8" t="s">
+        <v>234</v>
+      </c>
+      <c r="F8" t="s">
+        <v>234</v>
+      </c>
+      <c r="H8" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>240</v>
+      </c>
+      <c r="D9" t="s">
+        <v>235</v>
+      </c>
+      <c r="E9" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>240</v>
+      </c>
+      <c r="D10" t="s">
+        <v>234</v>
+      </c>
+      <c r="E10" t="s">
+        <v>234</v>
+      </c>
+      <c r="F10" t="s">
+        <v>234</v>
+      </c>
+      <c r="H10" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" t="s">
+        <v>240</v>
+      </c>
+      <c r="D11" t="s">
+        <v>235</v>
+      </c>
+      <c r="E11" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" t="s">
+        <v>240</v>
+      </c>
+      <c r="D12" t="s">
+        <v>234</v>
+      </c>
+      <c r="E12" t="s">
+        <v>234</v>
+      </c>
+      <c r="F12" t="s">
+        <v>234</v>
+      </c>
+      <c r="H12" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D13" t="s">
+        <v>235</v>
+      </c>
+      <c r="E13" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" t="s">
+        <v>240</v>
+      </c>
+      <c r="D14" t="s">
+        <v>234</v>
+      </c>
+      <c r="E14" t="s">
+        <v>234</v>
+      </c>
+      <c r="F14" t="s">
+        <v>234</v>
+      </c>
+      <c r="H14" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C15" t="s">
+        <v>240</v>
+      </c>
+      <c r="D15" t="s">
+        <v>235</v>
+      </c>
+      <c r="E15" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C16" t="s">
+        <v>240</v>
+      </c>
+      <c r="D16" t="s">
+        <v>234</v>
+      </c>
+      <c r="E16" t="s">
+        <v>234</v>
+      </c>
+      <c r="F16" t="s">
+        <v>234</v>
+      </c>
+      <c r="H16" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C17" t="s">
+        <v>240</v>
+      </c>
+      <c r="D17" t="s">
+        <v>235</v>
+      </c>
+      <c r="E17" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" t="s">
+        <v>240</v>
+      </c>
+      <c r="D18" t="s">
+        <v>234</v>
+      </c>
+      <c r="E18" t="s">
+        <v>234</v>
+      </c>
+      <c r="F18" t="s">
+        <v>234</v>
+      </c>
+      <c r="H18" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" t="s">
+        <v>240</v>
+      </c>
+      <c r="D19" t="s">
+        <v>235</v>
+      </c>
+      <c r="E19" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C20" t="s">
+        <v>240</v>
+      </c>
+      <c r="D20" t="s">
+        <v>234</v>
+      </c>
+      <c r="E20" t="s">
+        <v>234</v>
+      </c>
+      <c r="F20" t="s">
+        <v>234</v>
+      </c>
+      <c r="H20" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" t="s">
+        <v>240</v>
+      </c>
+      <c r="D21" t="s">
+        <v>235</v>
+      </c>
+      <c r="E21" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" t="s">
+        <v>240</v>
+      </c>
+      <c r="D22" t="s">
+        <v>234</v>
+      </c>
+      <c r="E22" t="s">
+        <v>234</v>
+      </c>
+      <c r="F22" t="s">
+        <v>234</v>
+      </c>
+      <c r="H22" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C23" t="s">
+        <v>240</v>
+      </c>
+      <c r="D23" t="s">
+        <v>235</v>
+      </c>
+      <c r="E23" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C24" t="s">
+        <v>240</v>
+      </c>
+      <c r="D24" t="s">
+        <v>234</v>
+      </c>
+      <c r="E24" t="s">
+        <v>234</v>
+      </c>
+      <c r="F24" t="s">
+        <v>234</v>
+      </c>
+      <c r="H24" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C25" t="s">
+        <v>240</v>
+      </c>
+      <c r="D25" t="s">
+        <v>235</v>
+      </c>
+      <c r="E25" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C26" t="s">
+        <v>240</v>
+      </c>
+      <c r="D26" t="s">
+        <v>234</v>
+      </c>
+      <c r="E26" t="s">
+        <v>234</v>
+      </c>
+      <c r="F26" t="s">
+        <v>234</v>
+      </c>
+      <c r="H26" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C27" t="s">
+        <v>240</v>
+      </c>
+      <c r="D27" t="s">
+        <v>235</v>
+      </c>
+      <c r="E27" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C28" t="s">
+        <v>240</v>
+      </c>
+      <c r="D28" t="s">
+        <v>234</v>
+      </c>
+      <c r="E28" t="s">
+        <v>234</v>
+      </c>
+      <c r="F28" t="s">
+        <v>234</v>
+      </c>
+      <c r="H28" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" t="s">
+        <v>240</v>
+      </c>
+      <c r="D29" t="s">
+        <v>235</v>
+      </c>
+      <c r="E29" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C30" t="s">
+        <v>240</v>
+      </c>
+      <c r="D30" t="s">
+        <v>234</v>
+      </c>
+      <c r="E30" t="s">
+        <v>234</v>
+      </c>
+      <c r="F30" t="s">
+        <v>234</v>
+      </c>
+      <c r="H30" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C31" t="s">
+        <v>240</v>
+      </c>
+      <c r="D31" t="s">
+        <v>235</v>
+      </c>
+      <c r="E31" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C32" t="s">
+        <v>240</v>
+      </c>
+      <c r="D32" t="s">
+        <v>234</v>
+      </c>
+      <c r="E32" t="s">
+        <v>234</v>
+      </c>
+      <c r="F32" t="s">
+        <v>234</v>
+      </c>
+      <c r="H32" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C33" t="s">
+        <v>240</v>
+      </c>
+      <c r="D33" t="s">
+        <v>235</v>
+      </c>
+      <c r="E33" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C34" t="s">
+        <v>240</v>
+      </c>
+      <c r="D34" t="s">
+        <v>234</v>
+      </c>
+      <c r="E34" t="s">
+        <v>234</v>
+      </c>
+      <c r="F34" t="s">
+        <v>234</v>
+      </c>
+      <c r="H34" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C35" t="s">
+        <v>240</v>
+      </c>
+      <c r="D35" t="s">
+        <v>235</v>
+      </c>
+      <c r="E35" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C36" t="s">
+        <v>240</v>
+      </c>
+      <c r="D36" t="s">
+        <v>234</v>
+      </c>
+      <c r="E36" t="s">
+        <v>234</v>
+      </c>
+      <c r="F36" t="s">
+        <v>234</v>
+      </c>
+      <c r="H36" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C37" t="s">
+        <v>240</v>
+      </c>
+      <c r="D37" t="s">
+        <v>235</v>
+      </c>
+      <c r="E37" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C38" t="s">
+        <v>240</v>
+      </c>
+      <c r="D38" t="s">
+        <v>234</v>
+      </c>
+      <c r="E38" t="s">
+        <v>234</v>
+      </c>
+      <c r="F38" t="s">
+        <v>234</v>
+      </c>
+      <c r="H38" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C39" t="s">
+        <v>240</v>
+      </c>
+      <c r="D39" t="s">
+        <v>235</v>
+      </c>
+      <c r="E39" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="C40" t="s">
+        <v>240</v>
+      </c>
+      <c r="D40" t="s">
+        <v>234</v>
+      </c>
+      <c r="E40" t="s">
+        <v>234</v>
+      </c>
+      <c r="F40" t="s">
+        <v>234</v>
+      </c>
+      <c r="H40" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C41" t="s">
+        <v>240</v>
+      </c>
+      <c r="D41" t="s">
+        <v>235</v>
+      </c>
+      <c r="E41" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C42" t="s">
+        <v>240</v>
+      </c>
+      <c r="D42" t="s">
+        <v>234</v>
+      </c>
+      <c r="E42" t="s">
+        <v>234</v>
+      </c>
+      <c r="F42" t="s">
+        <v>234</v>
+      </c>
+      <c r="H42" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C43" t="s">
+        <v>240</v>
+      </c>
+      <c r="D43" t="s">
+        <v>235</v>
+      </c>
+      <c r="E43" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C44" t="s">
+        <v>240</v>
+      </c>
+      <c r="D44" t="s">
+        <v>234</v>
+      </c>
+      <c r="E44" t="s">
+        <v>234</v>
+      </c>
+      <c r="F44" t="s">
+        <v>234</v>
+      </c>
+      <c r="H44" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C45" t="s">
+        <v>240</v>
+      </c>
+      <c r="D45" t="s">
+        <v>235</v>
+      </c>
+      <c r="E45" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C46" t="s">
+        <v>240</v>
+      </c>
+      <c r="D46" t="s">
+        <v>234</v>
+      </c>
+      <c r="E46" t="s">
+        <v>234</v>
+      </c>
+      <c r="F46" t="s">
+        <v>234</v>
+      </c>
+      <c r="H46" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C47" t="s">
+        <v>240</v>
+      </c>
+      <c r="D47" t="s">
+        <v>235</v>
+      </c>
+      <c r="E47" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C48" t="s">
+        <v>240</v>
+      </c>
+      <c r="D48" t="s">
+        <v>234</v>
+      </c>
+      <c r="E48" t="s">
+        <v>234</v>
+      </c>
+      <c r="F48" t="s">
+        <v>234</v>
+      </c>
+      <c r="H48" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C49" t="s">
+        <v>240</v>
+      </c>
+      <c r="D49" t="s">
+        <v>235</v>
+      </c>
+      <c r="E49" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C50" t="s">
+        <v>240</v>
+      </c>
+      <c r="D50" t="s">
+        <v>234</v>
+      </c>
+      <c r="E50" t="s">
+        <v>234</v>
+      </c>
+      <c r="F50" t="s">
+        <v>234</v>
+      </c>
+      <c r="H50" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C51" t="s">
+        <v>240</v>
+      </c>
+      <c r="D51" t="s">
+        <v>235</v>
+      </c>
+      <c r="E51" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="C52" t="s">
+        <v>240</v>
+      </c>
+      <c r="D52" t="s">
+        <v>234</v>
+      </c>
+      <c r="E52" t="s">
+        <v>234</v>
+      </c>
+      <c r="F52" t="s">
+        <v>234</v>
+      </c>
+      <c r="H52" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C53" t="s">
+        <v>240</v>
+      </c>
+      <c r="D53" t="s">
+        <v>235</v>
+      </c>
+      <c r="E53" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="C54" t="s">
+        <v>240</v>
+      </c>
+      <c r="D54" t="s">
+        <v>234</v>
+      </c>
+      <c r="E54" t="s">
+        <v>234</v>
+      </c>
+      <c r="F54" t="s">
+        <v>234</v>
+      </c>
+      <c r="H54" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C55" t="s">
+        <v>240</v>
+      </c>
+      <c r="D55" t="s">
+        <v>235</v>
+      </c>
+      <c r="E55" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C56" t="s">
+        <v>240</v>
+      </c>
+      <c r="D56" t="s">
+        <v>234</v>
+      </c>
+      <c r="E56" t="s">
+        <v>234</v>
+      </c>
+      <c r="F56" t="s">
+        <v>234</v>
+      </c>
+      <c r="H56" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C57" t="s">
+        <v>240</v>
+      </c>
+      <c r="D57" t="s">
+        <v>235</v>
+      </c>
+      <c r="E57" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C58" t="s">
+        <v>240</v>
+      </c>
+      <c r="D58" t="s">
+        <v>234</v>
+      </c>
+      <c r="E58" t="s">
+        <v>234</v>
+      </c>
+      <c r="F58" t="s">
+        <v>234</v>
+      </c>
+      <c r="H58" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C59" t="s">
+        <v>240</v>
+      </c>
+      <c r="D59" t="s">
+        <v>235</v>
+      </c>
+      <c r="E59" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C60" t="s">
+        <v>240</v>
+      </c>
+      <c r="D60" t="s">
+        <v>234</v>
+      </c>
+      <c r="E60" t="s">
+        <v>234</v>
+      </c>
+      <c r="F60" t="s">
+        <v>234</v>
+      </c>
+      <c r="H60" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C61" t="s">
+        <v>240</v>
+      </c>
+      <c r="D61" t="s">
+        <v>235</v>
+      </c>
+      <c r="E61" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="C62" t="s">
+        <v>240</v>
+      </c>
+      <c r="D62" t="s">
+        <v>234</v>
+      </c>
+      <c r="E62" t="s">
+        <v>234</v>
+      </c>
+      <c r="F62" t="s">
+        <v>234</v>
+      </c>
+      <c r="H62" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>157</v>
+      </c>
+      <c r="C63" t="s">
+        <v>240</v>
+      </c>
+      <c r="D63" t="s">
+        <v>235</v>
+      </c>
+      <c r="E63" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C64" t="s">
+        <v>240</v>
+      </c>
+      <c r="D64" t="s">
+        <v>234</v>
+      </c>
+      <c r="E64" t="s">
+        <v>234</v>
+      </c>
+      <c r="F64" t="s">
+        <v>234</v>
+      </c>
+      <c r="H64" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="C65" t="s">
+        <v>240</v>
+      </c>
+      <c r="D65" t="s">
+        <v>235</v>
+      </c>
+      <c r="E65" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="C66" t="s">
+        <v>240</v>
+      </c>
+      <c r="D66" t="s">
+        <v>234</v>
+      </c>
+      <c r="E66" t="s">
+        <v>234</v>
+      </c>
+      <c r="F66" t="s">
+        <v>234</v>
+      </c>
+      <c r="H66" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="C67" t="s">
+        <v>240</v>
+      </c>
+      <c r="D67" t="s">
+        <v>235</v>
+      </c>
+      <c r="E67" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
+        <v>166</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>167</v>
+      </c>
+      <c r="C68" t="s">
+        <v>240</v>
+      </c>
+      <c r="D68" t="s">
+        <v>234</v>
+      </c>
+      <c r="E68" t="s">
+        <v>234</v>
+      </c>
+      <c r="F68" t="s">
+        <v>234</v>
+      </c>
+      <c r="H68" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
+        <v>168</v>
+      </c>
+      <c r="B69" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C69" t="s">
+        <v>240</v>
+      </c>
+      <c r="D69" t="s">
+        <v>235</v>
+      </c>
+      <c r="E69" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
+        <v>170</v>
+      </c>
+      <c r="B70" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="C70" t="s">
+        <v>240</v>
+      </c>
+      <c r="D70" t="s">
+        <v>234</v>
+      </c>
+      <c r="E70" t="s">
+        <v>234</v>
+      </c>
+      <c r="F70" t="s">
+        <v>234</v>
+      </c>
+      <c r="H70" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="B71" s="2" t="s">
+        <v>173</v>
+      </c>
+      <c r="C71" t="s">
+        <v>240</v>
+      </c>
+      <c r="D71" t="s">
+        <v>235</v>
+      </c>
+      <c r="E71" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="B72" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C72" t="s">
+        <v>240</v>
+      </c>
+      <c r="D72" t="s">
+        <v>234</v>
+      </c>
+      <c r="E72" t="s">
+        <v>234</v>
+      </c>
+      <c r="F72" t="s">
+        <v>234</v>
+      </c>
+      <c r="H72" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="B73" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="C73" t="s">
+        <v>240</v>
+      </c>
+      <c r="D73" t="s">
+        <v>235</v>
+      </c>
+      <c r="E73" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A74" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="B74" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C74" t="s">
+        <v>240</v>
+      </c>
+      <c r="D74" t="s">
+        <v>234</v>
+      </c>
+      <c r="E74" t="s">
+        <v>234</v>
+      </c>
+      <c r="F74" t="s">
+        <v>234</v>
+      </c>
+      <c r="H74" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A75" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B75" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="C75" t="s">
+        <v>240</v>
+      </c>
+      <c r="D75" t="s">
+        <v>235</v>
+      </c>
+      <c r="E75" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A76" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="B76" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="C76" t="s">
+        <v>240</v>
+      </c>
+      <c r="D76" t="s">
+        <v>234</v>
+      </c>
+      <c r="E76" t="s">
+        <v>234</v>
+      </c>
+      <c r="F76" t="s">
+        <v>234</v>
+      </c>
+      <c r="H76" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A77" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="B77" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="C77" t="s">
+        <v>240</v>
+      </c>
+      <c r="D77" t="s">
+        <v>235</v>
+      </c>
+      <c r="E77" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A78" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B78" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="C78" t="s">
+        <v>240</v>
+      </c>
+      <c r="D78" t="s">
+        <v>234</v>
+      </c>
+      <c r="E78" t="s">
+        <v>234</v>
+      </c>
+      <c r="F78" t="s">
+        <v>234</v>
+      </c>
+      <c r="H78" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A79" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="B79" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C79" t="s">
+        <v>240</v>
+      </c>
+      <c r="D79" t="s">
+        <v>235</v>
+      </c>
+      <c r="E79" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A80" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="B80" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="C80" t="s">
+        <v>240</v>
+      </c>
+      <c r="D80" t="s">
+        <v>234</v>
+      </c>
+      <c r="E80" t="s">
+        <v>234</v>
+      </c>
+      <c r="F80" t="s">
+        <v>234</v>
+      </c>
+      <c r="H80" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A81" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="B81" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C81" t="s">
+        <v>240</v>
+      </c>
+      <c r="D81" t="s">
+        <v>235</v>
+      </c>
+      <c r="E81" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A82" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="B82" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="C82" t="s">
+        <v>240</v>
+      </c>
+      <c r="D82" t="s">
+        <v>234</v>
+      </c>
+      <c r="E82" t="s">
+        <v>234</v>
+      </c>
+      <c r="F82" t="s">
+        <v>234</v>
+      </c>
+      <c r="H82" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A83" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="B83" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="C83" t="s">
+        <v>240</v>
+      </c>
+      <c r="D83" t="s">
+        <v>235</v>
+      </c>
+      <c r="E83" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A84" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="B84" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="C84" t="s">
+        <v>240</v>
+      </c>
+      <c r="D84" t="s">
+        <v>234</v>
+      </c>
+      <c r="E84" t="s">
+        <v>234</v>
+      </c>
+      <c r="F84" t="s">
+        <v>234</v>
+      </c>
+      <c r="H84" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A85" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="B85" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="C85" t="s">
+        <v>240</v>
+      </c>
+      <c r="D85" t="s">
+        <v>235</v>
+      </c>
+      <c r="E85" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A86" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="B86" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="C86" t="s">
+        <v>240</v>
+      </c>
+      <c r="D86" t="s">
+        <v>234</v>
+      </c>
+      <c r="E86" t="s">
+        <v>234</v>
+      </c>
+      <c r="F86" t="s">
+        <v>234</v>
+      </c>
+      <c r="H86" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A87" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="B87" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="C87" t="s">
+        <v>240</v>
+      </c>
+      <c r="D87" t="s">
+        <v>235</v>
+      </c>
+      <c r="E87" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A88" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="B88" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="C88" t="s">
+        <v>240</v>
+      </c>
+      <c r="D88" t="s">
+        <v>234</v>
+      </c>
+      <c r="E88" t="s">
+        <v>234</v>
+      </c>
+      <c r="F88" t="s">
+        <v>234</v>
+      </c>
+      <c r="H88" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A89" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="B89" s="2" t="s">
+        <v>209</v>
+      </c>
+      <c r="C89" t="s">
+        <v>240</v>
+      </c>
+      <c r="D89" t="s">
+        <v>235</v>
+      </c>
+      <c r="E89" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A90" s="2" t="s">
+        <v>210</v>
+      </c>
+      <c r="B90" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="C90" t="s">
+        <v>240</v>
+      </c>
+      <c r="D90" t="s">
+        <v>234</v>
+      </c>
+      <c r="E90" t="s">
+        <v>234</v>
+      </c>
+      <c r="F90" t="s">
+        <v>234</v>
+      </c>
+      <c r="H90" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A91" s="2" t="s">
+        <v>212</v>
+      </c>
+      <c r="B91" s="2" t="s">
+        <v>213</v>
+      </c>
+      <c r="C91" t="s">
+        <v>240</v>
+      </c>
+      <c r="D91" t="s">
+        <v>235</v>
+      </c>
+      <c r="E91" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A92" s="2" t="s">
+        <v>214</v>
+      </c>
+      <c r="B92" s="2" t="s">
+        <v>215</v>
+      </c>
+      <c r="C92" t="s">
+        <v>240</v>
+      </c>
+      <c r="D92" t="s">
+        <v>234</v>
+      </c>
+      <c r="E92" t="s">
+        <v>234</v>
+      </c>
+      <c r="F92" t="s">
+        <v>234</v>
+      </c>
+      <c r="H92" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A93" s="2" t="s">
+        <v>216</v>
+      </c>
+      <c r="B93" s="2" t="s">
+        <v>217</v>
+      </c>
+      <c r="C93" t="s">
+        <v>240</v>
+      </c>
+      <c r="D93" t="s">
+        <v>235</v>
+      </c>
+      <c r="E93" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A94" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="B94" s="2" t="s">
+        <v>219</v>
+      </c>
+      <c r="C94" t="s">
+        <v>231</v>
+      </c>
+      <c r="D94" t="s">
+        <v>231</v>
+      </c>
+      <c r="E94" t="s">
+        <v>231</v>
+      </c>
+      <c r="F94" t="s">
+        <v>231</v>
+      </c>
+      <c r="H94" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A95" s="2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B95" s="2" t="s">
+        <v>221</v>
+      </c>
+      <c r="C95" t="s">
+        <v>231</v>
+      </c>
+      <c r="D95" t="s">
+        <v>231</v>
+      </c>
+      <c r="E95" t="s">
+        <v>231</v>
+      </c>
+      <c r="F95" t="s">
+        <v>231</v>
+      </c>
+      <c r="H95" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A96" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="B96" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="C96" t="s">
+        <v>231</v>
+      </c>
+      <c r="D96" t="s">
+        <v>231</v>
+      </c>
+      <c r="E96" t="s">
+        <v>231</v>
+      </c>
+      <c r="F96" t="s">
+        <v>231</v>
+      </c>
+      <c r="H96" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A97" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="B97" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="C97" t="s">
+        <v>231</v>
+      </c>
+      <c r="D97" t="s">
+        <v>231</v>
+      </c>
+      <c r="E97" t="s">
+        <v>231</v>
+      </c>
+      <c r="F97" t="s">
+        <v>231</v>
+      </c>
+      <c r="H97" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A98" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="B98" s="2" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A99" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="B99" s="2" t="s">
+        <v>229</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F99"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>